<commit_message>
Release V4 privacy mode and ranking improvements
</commit_message>
<xml_diff>
--- a/public/data/BMI ranking raw data.xlsx
+++ b/public/data/BMI ranking raw data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\bmi-ranking-app\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11A8E469-8B35-42D8-84D0-EC97B3CADF22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3F43146-0488-4DF5-A567-D7067FAAA913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BD8AD891-FD33-4205-9BBF-5D5C3ED867CE}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="55">
   <si>
     <t>名字</t>
   </si>
@@ -90,9 +90,6 @@
     <t>慧潔</t>
   </si>
   <si>
-    <t>*</t>
-  </si>
-  <si>
     <t>Charlene</t>
   </si>
   <si>
@@ -151,10 +148,6 @@
   </si>
   <si>
     <t>Kep</t>
-  </si>
-  <si>
-    <t>保密</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>Week1</t>
@@ -291,7 +284,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -308,6 +301,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -625,84 +621,84 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ACBC334-B2BB-40BA-ABE8-73477DDBF073}">
   <dimension ref="A1:L42"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="16.149999999999999" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C3" s="2">
         <v>160</v>
@@ -721,12 +717,12 @@
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
     </row>
-    <row r="4" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C4" s="2">
         <v>176</v>
@@ -745,12 +741,12 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C5" s="2">
         <v>175</v>
@@ -761,7 +757,9 @@
       <c r="E5" s="2">
         <v>74</v>
       </c>
-      <c r="F5" s="2"/>
+      <c r="F5" s="2">
+        <v>73.7</v>
+      </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -769,12 +767,12 @@
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
     </row>
-    <row r="6" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C6" s="2">
         <v>185</v>
@@ -793,12 +791,12 @@
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
     </row>
-    <row r="7" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A7" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C7" s="2">
         <v>172</v>
@@ -809,7 +807,9 @@
       <c r="E7" s="2">
         <v>68.2</v>
       </c>
-      <c r="F7" s="2"/>
+      <c r="F7" s="2">
+        <v>68.2</v>
+      </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
@@ -817,12 +817,12 @@
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
     </row>
-    <row r="8" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A8" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C8" s="2">
         <v>160</v>
@@ -833,7 +833,9 @@
       <c r="E8" s="2">
         <v>92.3</v>
       </c>
-      <c r="F8" s="2"/>
+      <c r="F8" s="2">
+        <v>92.7</v>
+      </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
@@ -841,12 +843,12 @@
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
     </row>
-    <row r="9" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C9" s="2">
         <v>175</v>
@@ -857,7 +859,9 @@
       <c r="E9" s="2">
         <v>84.1</v>
       </c>
-      <c r="F9" s="2"/>
+      <c r="F9" s="2">
+        <v>84.6</v>
+      </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -865,12 +869,12 @@
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
     </row>
-    <row r="10" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C10" s="2">
         <v>170</v>
@@ -889,12 +893,12 @@
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
     </row>
-    <row r="11" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C11" s="2">
         <v>180</v>
@@ -913,23 +917,17 @@
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
     </row>
-    <row r="12" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="F12" s="2"/>
+        <v>54</v>
+      </c>
+      <c r="C12" s="2"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="6"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -937,23 +935,17 @@
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
     </row>
-    <row r="13" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A13" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="F13" s="2"/>
+        <v>54</v>
+      </c>
+      <c r="C13" s="2"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="6"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
@@ -961,12 +953,12 @@
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
     </row>
-    <row r="14" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A14" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C14" s="2">
         <v>169</v>
@@ -977,7 +969,9 @@
       <c r="E14" s="2">
         <v>85.9</v>
       </c>
-      <c r="F14" s="2"/>
+      <c r="F14" s="2">
+        <v>84.6</v>
+      </c>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
@@ -985,12 +979,12 @@
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
     </row>
-    <row r="15" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A15" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C15" s="2">
         <v>166</v>
@@ -1001,7 +995,9 @@
       <c r="E15" s="2">
         <v>59.2</v>
       </c>
-      <c r="F15" s="2"/>
+      <c r="F15" s="2">
+        <v>59.2</v>
+      </c>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
@@ -1009,12 +1005,12 @@
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
     </row>
-    <row r="16" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A16" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C16" s="2">
         <v>170</v>
@@ -1025,7 +1021,9 @@
       <c r="E16" s="2">
         <v>80.3</v>
       </c>
-      <c r="F16" s="2"/>
+      <c r="F16" s="2">
+        <v>80.099999999999994</v>
+      </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
@@ -1033,12 +1031,12 @@
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
     </row>
-    <row r="17" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A17" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C17" s="2">
         <v>174</v>
@@ -1049,7 +1047,9 @@
       <c r="E17" s="2">
         <v>93.6</v>
       </c>
-      <c r="F17" s="2"/>
+      <c r="F17" s="2">
+        <v>94.9</v>
+      </c>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
@@ -1057,12 +1057,12 @@
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
     </row>
-    <row r="18" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A18" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C18" s="2">
         <v>188</v>
@@ -1073,7 +1073,9 @@
       <c r="E18" s="2">
         <v>88.2</v>
       </c>
-      <c r="F18" s="2"/>
+      <c r="F18" s="2">
+        <v>87.8</v>
+      </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
@@ -1081,12 +1083,12 @@
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
     </row>
-    <row r="19" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A19" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C19" s="2">
         <v>180</v>
@@ -1097,7 +1099,9 @@
       <c r="E19" s="2">
         <v>88.6</v>
       </c>
-      <c r="F19" s="2"/>
+      <c r="F19" s="2">
+        <v>88.5</v>
+      </c>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
@@ -1105,12 +1109,12 @@
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
     </row>
-    <row r="20" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A20" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C20" s="2">
         <v>177</v>
@@ -1121,7 +1125,9 @@
       <c r="E20" s="2">
         <v>90</v>
       </c>
-      <c r="F20" s="2"/>
+      <c r="F20" s="2">
+        <v>89.8</v>
+      </c>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
@@ -1129,12 +1135,12 @@
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
     </row>
-    <row r="21" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A21" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C21" s="2">
         <v>177</v>
@@ -1153,12 +1159,12 @@
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
     </row>
-    <row r="22" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A22" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C22" s="2">
         <v>181</v>
@@ -1169,7 +1175,9 @@
       <c r="E22" s="2">
         <v>83.9</v>
       </c>
-      <c r="F22" s="2"/>
+      <c r="F22" s="2">
+        <v>83.3</v>
+      </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
@@ -1177,12 +1185,12 @@
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
     </row>
-    <row r="23" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A23" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C23" s="2">
         <v>186</v>
@@ -1193,7 +1201,9 @@
       <c r="E23" s="2">
         <v>115.1</v>
       </c>
-      <c r="F23" s="2"/>
+      <c r="F23" s="2">
+        <v>114.2</v>
+      </c>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
@@ -1201,12 +1211,12 @@
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
     </row>
-    <row r="24" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A24" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C24" s="2">
         <v>180</v>
@@ -1217,7 +1227,9 @@
       <c r="E24" s="2">
         <v>106.9</v>
       </c>
-      <c r="F24" s="2"/>
+      <c r="F24" s="2">
+        <v>106.1</v>
+      </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
@@ -1225,12 +1237,12 @@
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
     </row>
-    <row r="25" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A25" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C25" s="2">
         <v>172</v>
@@ -1241,7 +1253,9 @@
       <c r="E25" s="2">
         <v>67.599999999999994</v>
       </c>
-      <c r="F25" s="2"/>
+      <c r="F25" s="2">
+        <v>67.2</v>
+      </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
@@ -1249,12 +1263,12 @@
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
     </row>
-    <row r="26" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A26" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C26" s="2">
         <v>174.5</v>
@@ -1265,7 +1279,9 @@
       <c r="E26" s="2">
         <v>63.1</v>
       </c>
-      <c r="F26" s="2"/>
+      <c r="F26" s="2">
+        <v>63</v>
+      </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
@@ -1273,12 +1289,12 @@
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
     </row>
-    <row r="27" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A27" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C27" s="2">
         <v>163</v>
@@ -1289,7 +1305,9 @@
       <c r="E27" s="2">
         <v>80.8</v>
       </c>
-      <c r="F27" s="2"/>
+      <c r="F27" s="2">
+        <v>80.900000000000006</v>
+      </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
@@ -1297,12 +1315,12 @@
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
     </row>
-    <row r="28" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A28" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C28" s="2">
         <v>164</v>
@@ -1321,12 +1339,12 @@
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
     </row>
-    <row r="29" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A29" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C29" s="2">
         <v>177</v>
@@ -1345,12 +1363,12 @@
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
     </row>
-    <row r="30" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A30" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C30" s="2">
         <v>167</v>
@@ -1369,12 +1387,12 @@
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
     </row>
-    <row r="31" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A31" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C31" s="2">
         <v>178</v>
@@ -1385,7 +1403,9 @@
       <c r="E31" s="2">
         <v>112.2</v>
       </c>
-      <c r="F31" s="2"/>
+      <c r="F31" s="2">
+        <v>110.1</v>
+      </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
@@ -1393,12 +1413,12 @@
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
     </row>
-    <row r="32" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A32" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C32" s="2">
         <v>171</v>
@@ -1409,7 +1429,9 @@
       <c r="E32" s="2">
         <v>74.2</v>
       </c>
-      <c r="F32" s="2"/>
+      <c r="F32" s="2">
+        <v>75.3</v>
+      </c>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
@@ -1417,12 +1439,12 @@
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
     </row>
-    <row r="33" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A33" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C33" s="2">
         <v>180</v>
@@ -1433,7 +1455,9 @@
       <c r="E33" s="2">
         <v>87.2</v>
       </c>
-      <c r="F33" s="2"/>
+      <c r="F33" s="2">
+        <v>86.8</v>
+      </c>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
@@ -1441,12 +1465,12 @@
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
     </row>
-    <row r="34" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A34" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C34" s="2">
         <v>168</v>
@@ -1457,7 +1481,9 @@
       <c r="E34" s="2">
         <v>71.099999999999994</v>
       </c>
-      <c r="F34" s="2"/>
+      <c r="F34" s="2">
+        <v>71.2</v>
+      </c>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
@@ -1465,12 +1491,12 @@
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>
     </row>
-    <row r="35" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A35" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C35" s="2">
         <v>169</v>
@@ -1481,7 +1507,9 @@
       <c r="E35" s="2">
         <v>64.400000000000006</v>
       </c>
-      <c r="F35" s="2"/>
+      <c r="F35" s="2">
+        <v>64.8</v>
+      </c>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
@@ -1489,12 +1517,12 @@
       <c r="K35" s="2"/>
       <c r="L35" s="2"/>
     </row>
-    <row r="36" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A36" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C36" s="2">
         <v>177</v>
@@ -1505,7 +1533,9 @@
       <c r="E36" s="2">
         <v>73</v>
       </c>
-      <c r="F36" s="2"/>
+      <c r="F36" s="2">
+        <v>74</v>
+      </c>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
@@ -1513,12 +1543,12 @@
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
     </row>
-    <row r="37" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A37" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C37" s="2">
         <v>170</v>
@@ -1529,7 +1559,9 @@
       <c r="E37" s="2">
         <v>82.6</v>
       </c>
-      <c r="F37" s="2"/>
+      <c r="F37" s="2">
+        <v>82.5</v>
+      </c>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
@@ -1537,12 +1569,12 @@
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
     </row>
-    <row r="38" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C38" s="3">
         <v>171</v>
@@ -1561,12 +1593,12 @@
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
     </row>
-    <row r="39" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C39" s="3">
         <v>177</v>
@@ -1585,12 +1617,12 @@
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
     </row>
-    <row r="40" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C40" s="3">
         <v>183</v>
@@ -1609,12 +1641,12 @@
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
     </row>
-    <row r="41" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C41" s="3">
         <v>176</v>
@@ -1633,12 +1665,12 @@
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
     </row>
-    <row r="42" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C42" s="3">
         <v>172</v>
@@ -1649,7 +1681,9 @@
       <c r="E42" s="3">
         <v>72</v>
       </c>
-      <c r="F42" s="3"/>
+      <c r="F42" s="3">
+        <v>72.599999999999994</v>
+      </c>
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
       <c r="I42" s="3"/>

</xml_diff>

<commit_message>
Update Week4 ranking data
</commit_message>
<xml_diff>
--- a/public/data/BMI ranking raw data.xlsx
+++ b/public/data/BMI ranking raw data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\bmi-ranking-app\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3F43146-0488-4DF5-A567-D7067FAAA913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5D0B6EE-55A2-435A-9668-6F335369CB48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BD8AD891-FD33-4205-9BBF-5D5C3ED867CE}"/>
   </bookViews>
@@ -710,7 +710,9 @@
         <v>68</v>
       </c>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2">
+        <v>67.8</v>
+      </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
@@ -734,7 +736,9 @@
         <v>68.8</v>
       </c>
       <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
+      <c r="G4" s="2">
+        <v>68</v>
+      </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
@@ -760,7 +764,9 @@
       <c r="F5" s="2">
         <v>73.7</v>
       </c>
-      <c r="G5" s="2"/>
+      <c r="G5" s="2">
+        <v>74.099999999999994</v>
+      </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -784,7 +790,9 @@
         <v>78.599999999999994</v>
       </c>
       <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
+      <c r="G6" s="2">
+        <v>78.599999999999994</v>
+      </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
@@ -810,7 +818,9 @@
       <c r="F7" s="2">
         <v>68.2</v>
       </c>
-      <c r="G7" s="2"/>
+      <c r="G7" s="2">
+        <v>67.8</v>
+      </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
@@ -836,7 +846,9 @@
       <c r="F8" s="2">
         <v>92.7</v>
       </c>
-      <c r="G8" s="2"/>
+      <c r="G8" s="2">
+        <v>91.9</v>
+      </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -862,7 +874,9 @@
       <c r="F9" s="2">
         <v>84.6</v>
       </c>
-      <c r="G9" s="2"/>
+      <c r="G9" s="2">
+        <v>84.6</v>
+      </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -886,7 +900,9 @@
         <v>70.8</v>
       </c>
       <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
+      <c r="G10" s="2">
+        <v>70.8</v>
+      </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
@@ -910,7 +926,9 @@
         <v>138</v>
       </c>
       <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
+      <c r="G11" s="2">
+        <v>138</v>
+      </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -972,7 +990,9 @@
       <c r="F14" s="2">
         <v>84.6</v>
       </c>
-      <c r="G14" s="2"/>
+      <c r="G14" s="2">
+        <v>84.6</v>
+      </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
@@ -998,7 +1018,9 @@
       <c r="F15" s="2">
         <v>59.2</v>
       </c>
-      <c r="G15" s="2"/>
+      <c r="G15" s="2">
+        <v>59.2</v>
+      </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
@@ -1024,7 +1046,9 @@
       <c r="F16" s="2">
         <v>80.099999999999994</v>
       </c>
-      <c r="G16" s="2"/>
+      <c r="G16" s="2">
+        <v>80.099999999999994</v>
+      </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -1050,7 +1074,9 @@
       <c r="F17" s="2">
         <v>94.9</v>
       </c>
-      <c r="G17" s="2"/>
+      <c r="G17" s="2">
+        <v>93.2</v>
+      </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -1076,7 +1102,9 @@
       <c r="F18" s="2">
         <v>87.8</v>
       </c>
-      <c r="G18" s="2"/>
+      <c r="G18" s="2">
+        <v>88.5</v>
+      </c>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -1102,7 +1130,9 @@
       <c r="F19" s="2">
         <v>88.5</v>
       </c>
-      <c r="G19" s="2"/>
+      <c r="G19" s="2">
+        <v>87.8</v>
+      </c>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -1128,7 +1158,9 @@
       <c r="F20" s="2">
         <v>89.8</v>
       </c>
-      <c r="G20" s="2"/>
+      <c r="G20" s="2">
+        <v>88.6</v>
+      </c>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
@@ -1152,7 +1184,9 @@
         <v>71.7</v>
       </c>
       <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+      <c r="G21" s="2">
+        <v>70.400000000000006</v>
+      </c>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -1178,7 +1212,9 @@
       <c r="F22" s="2">
         <v>83.3</v>
       </c>
-      <c r="G22" s="2"/>
+      <c r="G22" s="2">
+        <v>85.1</v>
+      </c>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
@@ -1204,7 +1240,9 @@
       <c r="F23" s="2">
         <v>114.2</v>
       </c>
-      <c r="G23" s="2"/>
+      <c r="G23" s="2">
+        <v>114.6</v>
+      </c>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
@@ -1230,7 +1268,9 @@
       <c r="F24" s="2">
         <v>106.1</v>
       </c>
-      <c r="G24" s="2"/>
+      <c r="G24" s="2">
+        <v>106.1</v>
+      </c>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
@@ -1256,7 +1296,9 @@
       <c r="F25" s="2">
         <v>67.2</v>
       </c>
-      <c r="G25" s="2"/>
+      <c r="G25" s="2">
+        <v>67.7</v>
+      </c>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
@@ -1282,7 +1324,9 @@
       <c r="F26" s="2">
         <v>63</v>
       </c>
-      <c r="G26" s="2"/>
+      <c r="G26" s="2">
+        <v>62.8</v>
+      </c>
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
@@ -1308,7 +1352,9 @@
       <c r="F27" s="2">
         <v>80.900000000000006</v>
       </c>
-      <c r="G27" s="2"/>
+      <c r="G27" s="2">
+        <v>79.400000000000006</v>
+      </c>
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
@@ -1332,7 +1378,9 @@
         <v>74.8</v>
       </c>
       <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
+      <c r="G28" s="2">
+        <v>74.8</v>
+      </c>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
@@ -1356,7 +1404,9 @@
         <v>90.1</v>
       </c>
       <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
+      <c r="G29" s="2">
+        <v>90.1</v>
+      </c>
       <c r="H29" s="2"/>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
@@ -1380,7 +1430,9 @@
         <v>78</v>
       </c>
       <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
+      <c r="G30" s="2">
+        <v>78</v>
+      </c>
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
@@ -1406,7 +1458,9 @@
       <c r="F31" s="2">
         <v>110.1</v>
       </c>
-      <c r="G31" s="2"/>
+      <c r="G31" s="2">
+        <v>107.8</v>
+      </c>
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
@@ -1432,7 +1486,9 @@
       <c r="F32" s="2">
         <v>75.3</v>
       </c>
-      <c r="G32" s="2"/>
+      <c r="G32" s="2">
+        <v>74.599999999999994</v>
+      </c>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
@@ -1458,7 +1514,9 @@
       <c r="F33" s="2">
         <v>86.8</v>
       </c>
-      <c r="G33" s="2"/>
+      <c r="G33" s="2">
+        <v>86.8</v>
+      </c>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
@@ -1484,7 +1542,9 @@
       <c r="F34" s="2">
         <v>71.2</v>
       </c>
-      <c r="G34" s="2"/>
+      <c r="G34" s="2">
+        <v>71.5</v>
+      </c>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
@@ -1510,7 +1570,9 @@
       <c r="F35" s="2">
         <v>64.8</v>
       </c>
-      <c r="G35" s="2"/>
+      <c r="G35" s="2">
+        <v>65.5</v>
+      </c>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
@@ -1536,7 +1598,9 @@
       <c r="F36" s="2">
         <v>74</v>
       </c>
-      <c r="G36" s="2"/>
+      <c r="G36" s="2">
+        <v>73.599999999999994</v>
+      </c>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
@@ -1562,7 +1626,9 @@
       <c r="F37" s="2">
         <v>82.5</v>
       </c>
-      <c r="G37" s="2"/>
+      <c r="G37" s="2">
+        <v>82.6</v>
+      </c>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
@@ -1586,7 +1652,9 @@
         <v>89.4</v>
       </c>
       <c r="F38" s="3"/>
-      <c r="G38" s="3"/>
+      <c r="G38" s="3">
+        <v>89.4</v>
+      </c>
       <c r="H38" s="3"/>
       <c r="I38" s="3"/>
       <c r="J38" s="3"/>
@@ -1610,7 +1678,9 @@
         <v>79.599999999999994</v>
       </c>
       <c r="F39" s="3"/>
-      <c r="G39" s="3"/>
+      <c r="G39" s="3">
+        <v>79.599999999999994</v>
+      </c>
       <c r="H39" s="3"/>
       <c r="I39" s="3"/>
       <c r="J39" s="3"/>
@@ -1634,7 +1704,9 @@
         <v>93.6</v>
       </c>
       <c r="F40" s="3"/>
-      <c r="G40" s="3"/>
+      <c r="G40" s="3">
+        <v>93.6</v>
+      </c>
       <c r="H40" s="3"/>
       <c r="I40" s="3"/>
       <c r="J40" s="3"/>
@@ -1658,7 +1730,9 @@
         <v>94.8</v>
       </c>
       <c r="F41" s="3"/>
-      <c r="G41" s="3"/>
+      <c r="G41" s="3">
+        <v>94.8</v>
+      </c>
       <c r="H41" s="3"/>
       <c r="I41" s="3"/>
       <c r="J41" s="3"/>
@@ -1684,7 +1758,9 @@
       <c r="F42" s="3">
         <v>72.599999999999994</v>
       </c>
-      <c r="G42" s="3"/>
+      <c r="G42" s="3">
+        <v>70.599999999999994</v>
+      </c>
       <c r="H42" s="3"/>
       <c r="I42" s="3"/>
       <c r="J42" s="3"/>

</xml_diff>

<commit_message>
Update Week5 ranking data
</commit_message>
<xml_diff>
--- a/public/data/BMI ranking raw data.xlsx
+++ b/public/data/BMI ranking raw data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\bmi-ranking-app\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5D0B6EE-55A2-435A-9668-6F335369CB48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{623E41CF-7956-41D2-B50A-4700FBC5F67E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BD8AD891-FD33-4205-9BBF-5D5C3ED867CE}"/>
   </bookViews>
@@ -284,7 +284,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -304,6 +304,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -621,9 +624,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ACBC334-B2BB-40BA-ABE8-73477DDBF073}">
   <dimension ref="A1:L42"/>
-  <sheetFormatPr defaultRowHeight="16.149999999999999" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="8.5" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -655,7 +661,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -693,7 +699,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -713,13 +719,15 @@
       <c r="G3" s="2">
         <v>67.8</v>
       </c>
-      <c r="H3" s="2"/>
+      <c r="H3" s="2">
+        <v>66.7</v>
+      </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
     </row>
-    <row r="4" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -739,13 +747,15 @@
       <c r="G4" s="2">
         <v>68</v>
       </c>
-      <c r="H4" s="2"/>
+      <c r="H4" s="2">
+        <v>68</v>
+      </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -767,13 +777,15 @@
       <c r="G5" s="2">
         <v>74.099999999999994</v>
       </c>
-      <c r="H5" s="2"/>
+      <c r="H5" s="2">
+        <v>74.099999999999994</v>
+      </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
     </row>
-    <row r="6" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -793,13 +805,15 @@
       <c r="G6" s="2">
         <v>78.599999999999994</v>
       </c>
-      <c r="H6" s="2"/>
+      <c r="H6" s="2">
+        <v>78.599999999999994</v>
+      </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
     </row>
-    <row r="7" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>15</v>
       </c>
@@ -821,13 +835,15 @@
       <c r="G7" s="2">
         <v>67.8</v>
       </c>
-      <c r="H7" s="2"/>
+      <c r="H7" s="2">
+        <v>67.8</v>
+      </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
     </row>
-    <row r="8" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>16</v>
       </c>
@@ -849,13 +865,15 @@
       <c r="G8" s="2">
         <v>91.9</v>
       </c>
-      <c r="H8" s="2"/>
+      <c r="H8" s="2">
+        <v>91.7</v>
+      </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
     </row>
-    <row r="9" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
@@ -877,13 +895,15 @@
       <c r="G9" s="2">
         <v>84.6</v>
       </c>
-      <c r="H9" s="2"/>
+      <c r="H9" s="2">
+        <v>85.2</v>
+      </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
     </row>
-    <row r="10" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
@@ -903,13 +923,15 @@
       <c r="G10" s="2">
         <v>70.8</v>
       </c>
-      <c r="H10" s="2"/>
+      <c r="H10" s="2">
+        <v>70.7</v>
+      </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
     </row>
-    <row r="11" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -929,13 +951,15 @@
       <c r="G11" s="2">
         <v>138</v>
       </c>
-      <c r="H11" s="2"/>
+      <c r="H11" s="2">
+        <v>138</v>
+      </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
     </row>
-    <row r="12" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -944,16 +968,16 @@
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+      <c r="E12" s="7"/>
       <c r="F12" s="6"/>
-      <c r="G12" s="2"/>
+      <c r="G12" s="6"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
     </row>
-    <row r="13" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>21</v>
       </c>
@@ -971,7 +995,7 @@
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
     </row>
-    <row r="14" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -993,13 +1017,15 @@
       <c r="G14" s="2">
         <v>84.6</v>
       </c>
-      <c r="H14" s="2"/>
+      <c r="H14" s="2">
+        <v>83.8</v>
+      </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
     </row>
-    <row r="15" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1021,13 +1047,15 @@
       <c r="G15" s="2">
         <v>59.2</v>
       </c>
-      <c r="H15" s="2"/>
+      <c r="H15" s="2">
+        <v>59.2</v>
+      </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
     </row>
-    <row r="16" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>24</v>
       </c>
@@ -1049,13 +1077,15 @@
       <c r="G16" s="2">
         <v>80.099999999999994</v>
       </c>
-      <c r="H16" s="2"/>
+      <c r="H16" s="2">
+        <v>79</v>
+      </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
     </row>
-    <row r="17" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>25</v>
       </c>
@@ -1077,13 +1107,15 @@
       <c r="G17" s="2">
         <v>93.2</v>
       </c>
-      <c r="H17" s="2"/>
+      <c r="H17" s="2">
+        <v>93.2</v>
+      </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
     </row>
-    <row r="18" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>26</v>
       </c>
@@ -1105,13 +1137,15 @@
       <c r="G18" s="2">
         <v>88.5</v>
       </c>
-      <c r="H18" s="2"/>
+      <c r="H18" s="2">
+        <v>87.9</v>
+      </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
     </row>
-    <row r="19" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>27</v>
       </c>
@@ -1133,13 +1167,15 @@
       <c r="G19" s="2">
         <v>87.8</v>
       </c>
-      <c r="H19" s="2"/>
+      <c r="H19" s="2">
+        <v>87.7</v>
+      </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
     </row>
-    <row r="20" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>28</v>
       </c>
@@ -1161,13 +1197,15 @@
       <c r="G20" s="2">
         <v>88.6</v>
       </c>
-      <c r="H20" s="2"/>
+      <c r="H20" s="2">
+        <v>83.8</v>
+      </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
     </row>
-    <row r="21" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>6</v>
       </c>
@@ -1187,13 +1225,15 @@
       <c r="G21" s="2">
         <v>70.400000000000006</v>
       </c>
-      <c r="H21" s="2"/>
+      <c r="H21" s="2">
+        <v>70.7</v>
+      </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
     </row>
-    <row r="22" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>7</v>
       </c>
@@ -1215,13 +1255,15 @@
       <c r="G22" s="2">
         <v>85.1</v>
       </c>
-      <c r="H22" s="2"/>
+      <c r="H22" s="2">
+        <v>84.1</v>
+      </c>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
     </row>
-    <row r="23" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>8</v>
       </c>
@@ -1243,13 +1285,15 @@
       <c r="G23" s="2">
         <v>114.6</v>
       </c>
-      <c r="H23" s="2"/>
+      <c r="H23" s="2">
+        <v>111</v>
+      </c>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
     </row>
-    <row r="24" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="24" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>9</v>
       </c>
@@ -1271,13 +1315,15 @@
       <c r="G24" s="2">
         <v>106.1</v>
       </c>
-      <c r="H24" s="2"/>
+      <c r="H24" s="2">
+        <v>106.1</v>
+      </c>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
     </row>
-    <row r="25" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>10</v>
       </c>
@@ -1299,13 +1345,15 @@
       <c r="G25" s="2">
         <v>67.7</v>
       </c>
-      <c r="H25" s="2"/>
+      <c r="H25" s="2">
+        <v>67.2</v>
+      </c>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
     </row>
-    <row r="26" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>11</v>
       </c>
@@ -1327,13 +1375,15 @@
       <c r="G26" s="2">
         <v>62.8</v>
       </c>
-      <c r="H26" s="2"/>
+      <c r="H26" s="2">
+        <v>62.5</v>
+      </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
     </row>
-    <row r="27" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>29</v>
       </c>
@@ -1355,13 +1405,15 @@
       <c r="G27" s="2">
         <v>79.400000000000006</v>
       </c>
-      <c r="H27" s="2"/>
+      <c r="H27" s="2">
+        <v>77.5</v>
+      </c>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
     </row>
-    <row r="28" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>30</v>
       </c>
@@ -1381,13 +1433,15 @@
       <c r="G28" s="2">
         <v>74.8</v>
       </c>
-      <c r="H28" s="2"/>
+      <c r="H28" s="2">
+        <v>74.8</v>
+      </c>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
     </row>
-    <row r="29" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>31</v>
       </c>
@@ -1407,13 +1461,15 @@
       <c r="G29" s="2">
         <v>90.1</v>
       </c>
-      <c r="H29" s="2"/>
+      <c r="H29" s="2">
+        <v>90</v>
+      </c>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
     </row>
-    <row r="30" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>32</v>
       </c>
@@ -1433,13 +1489,15 @@
       <c r="G30" s="2">
         <v>78</v>
       </c>
-      <c r="H30" s="2"/>
+      <c r="H30" s="2">
+        <v>78</v>
+      </c>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
     </row>
-    <row r="31" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>33</v>
       </c>
@@ -1461,13 +1519,15 @@
       <c r="G31" s="2">
         <v>107.8</v>
       </c>
-      <c r="H31" s="2"/>
+      <c r="H31" s="2">
+        <v>106.5</v>
+      </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
     </row>
-    <row r="32" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="32" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>34</v>
       </c>
@@ -1489,13 +1549,15 @@
       <c r="G32" s="2">
         <v>74.599999999999994</v>
       </c>
-      <c r="H32" s="2"/>
+      <c r="H32" s="2">
+        <v>74.3</v>
+      </c>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
     </row>
-    <row r="33" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="33" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>35</v>
       </c>
@@ -1517,13 +1579,15 @@
       <c r="G33" s="2">
         <v>86.8</v>
       </c>
-      <c r="H33" s="2"/>
+      <c r="H33" s="2">
+        <v>88.2</v>
+      </c>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
     </row>
-    <row r="34" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="34" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>36</v>
       </c>
@@ -1545,13 +1609,15 @@
       <c r="G34" s="2">
         <v>71.5</v>
       </c>
-      <c r="H34" s="2"/>
+      <c r="H34" s="2">
+        <v>71.5</v>
+      </c>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>
     </row>
-    <row r="35" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="35" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>12</v>
       </c>
@@ -1573,13 +1639,15 @@
       <c r="G35" s="2">
         <v>65.5</v>
       </c>
-      <c r="H35" s="2"/>
+      <c r="H35" s="2">
+        <v>65.2</v>
+      </c>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
       <c r="L35" s="2"/>
     </row>
-    <row r="36" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="36" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>13</v>
       </c>
@@ -1601,13 +1669,15 @@
       <c r="G36" s="2">
         <v>73.599999999999994</v>
       </c>
-      <c r="H36" s="2"/>
+      <c r="H36" s="2">
+        <v>73</v>
+      </c>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
     </row>
-    <row r="37" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="37" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>14</v>
       </c>
@@ -1629,13 +1699,15 @@
       <c r="G37" s="2">
         <v>82.6</v>
       </c>
-      <c r="H37" s="2"/>
+      <c r="H37" s="2">
+        <v>83.3</v>
+      </c>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
     </row>
-    <row r="38" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>37</v>
       </c>
@@ -1655,13 +1727,15 @@
       <c r="G38" s="3">
         <v>89.4</v>
       </c>
-      <c r="H38" s="3"/>
+      <c r="H38" s="3">
+        <v>89.4</v>
+      </c>
       <c r="I38" s="3"/>
       <c r="J38" s="3"/>
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
     </row>
-    <row r="39" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>38</v>
       </c>
@@ -1681,13 +1755,15 @@
       <c r="G39" s="3">
         <v>79.599999999999994</v>
       </c>
-      <c r="H39" s="3"/>
+      <c r="H39" s="3">
+        <v>79.599999999999994</v>
+      </c>
       <c r="I39" s="3"/>
       <c r="J39" s="3"/>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
     </row>
-    <row r="40" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>39</v>
       </c>
@@ -1707,13 +1783,15 @@
       <c r="G40" s="3">
         <v>93.6</v>
       </c>
-      <c r="H40" s="3"/>
+      <c r="H40" s="3">
+        <v>93.6</v>
+      </c>
       <c r="I40" s="3"/>
       <c r="J40" s="3"/>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
     </row>
-    <row r="41" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>40</v>
       </c>
@@ -1733,13 +1811,15 @@
       <c r="G41" s="3">
         <v>94.8</v>
       </c>
-      <c r="H41" s="3"/>
+      <c r="H41" s="3">
+        <v>94.8</v>
+      </c>
       <c r="I41" s="3"/>
       <c r="J41" s="3"/>
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
     </row>
-    <row r="42" spans="1:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>51</v>
       </c>
@@ -1761,7 +1841,9 @@
       <c r="G42" s="3">
         <v>70.599999999999994</v>
       </c>
-      <c r="H42" s="3"/>
+      <c r="H42" s="3">
+        <v>71.3</v>
+      </c>
       <c r="I42" s="3"/>
       <c r="J42" s="3"/>
       <c r="K42" s="3"/>

</xml_diff>

<commit_message>
Update Week6 ranking data
</commit_message>
<xml_diff>
--- a/public/data/BMI ranking raw data.xlsx
+++ b/public/data/BMI ranking raw data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\bmi-ranking-app\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{623E41CF-7956-41D2-B50A-4700FBC5F67E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F1035B7-1088-4179-AD91-01392FE42341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BD8AD891-FD33-4205-9BBF-5D5C3ED867CE}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="56">
   <si>
     <t>名字</t>
   </si>
@@ -196,6 +196,9 @@
   <si>
     <t>F</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>*</t>
   </si>
 </sst>
 </file>
@@ -722,7 +725,9 @@
       <c r="H3" s="2">
         <v>66.7</v>
       </c>
-      <c r="I3" s="2"/>
+      <c r="I3" s="2">
+        <v>65.7</v>
+      </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
@@ -750,7 +755,9 @@
       <c r="H4" s="2">
         <v>68</v>
       </c>
-      <c r="I4" s="2"/>
+      <c r="I4" s="2">
+        <v>68</v>
+      </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -780,7 +787,9 @@
       <c r="H5" s="2">
         <v>74.099999999999994</v>
       </c>
-      <c r="I5" s="2"/>
+      <c r="I5" s="2">
+        <v>73.7</v>
+      </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -808,7 +817,9 @@
       <c r="H6" s="2">
         <v>78.599999999999994</v>
       </c>
-      <c r="I6" s="2"/>
+      <c r="I6" s="2">
+        <v>78.599999999999994</v>
+      </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
@@ -838,7 +849,9 @@
       <c r="H7" s="2">
         <v>67.8</v>
       </c>
-      <c r="I7" s="2"/>
+      <c r="I7" s="2">
+        <v>67.8</v>
+      </c>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
@@ -868,7 +881,9 @@
       <c r="H8" s="2">
         <v>91.7</v>
       </c>
-      <c r="I8" s="2"/>
+      <c r="I8" s="2">
+        <v>91.7</v>
+      </c>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
@@ -898,7 +913,9 @@
       <c r="H9" s="2">
         <v>85.2</v>
       </c>
-      <c r="I9" s="2"/>
+      <c r="I9" s="2">
+        <v>85.2</v>
+      </c>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
@@ -926,7 +943,9 @@
       <c r="H10" s="2">
         <v>70.7</v>
       </c>
-      <c r="I10" s="2"/>
+      <c r="I10" s="2">
+        <v>70.7</v>
+      </c>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
@@ -954,7 +973,9 @@
       <c r="H11" s="2">
         <v>138</v>
       </c>
-      <c r="I11" s="2"/>
+      <c r="I11" s="2">
+        <v>138</v>
+      </c>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
@@ -972,7 +993,9 @@
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
       <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
+      <c r="I12" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
@@ -990,7 +1013,9 @@
       <c r="F13" s="6"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
+      <c r="I13" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
@@ -1020,7 +1045,9 @@
       <c r="H14" s="2">
         <v>83.8</v>
       </c>
-      <c r="I14" s="2"/>
+      <c r="I14" s="2">
+        <v>82.5</v>
+      </c>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
@@ -1050,7 +1077,9 @@
       <c r="H15" s="2">
         <v>59.2</v>
       </c>
-      <c r="I15" s="2"/>
+      <c r="I15" s="2">
+        <v>59.2</v>
+      </c>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
@@ -1080,7 +1109,9 @@
       <c r="H16" s="2">
         <v>79</v>
       </c>
-      <c r="I16" s="2"/>
+      <c r="I16" s="2">
+        <v>79</v>
+      </c>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
@@ -1110,7 +1141,9 @@
       <c r="H17" s="2">
         <v>93.2</v>
       </c>
-      <c r="I17" s="2"/>
+      <c r="I17" s="2">
+        <v>93.9</v>
+      </c>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
@@ -1140,7 +1173,9 @@
       <c r="H18" s="2">
         <v>87.9</v>
       </c>
-      <c r="I18" s="2"/>
+      <c r="I18" s="2">
+        <v>87.9</v>
+      </c>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
@@ -1170,7 +1205,9 @@
       <c r="H19" s="2">
         <v>87.7</v>
       </c>
-      <c r="I19" s="2"/>
+      <c r="I19" s="2">
+        <v>87</v>
+      </c>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
@@ -1200,7 +1237,9 @@
       <c r="H20" s="2">
         <v>83.8</v>
       </c>
-      <c r="I20" s="2"/>
+      <c r="I20" s="2">
+        <v>84.9</v>
+      </c>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
@@ -1228,7 +1267,9 @@
       <c r="H21" s="2">
         <v>70.7</v>
       </c>
-      <c r="I21" s="2"/>
+      <c r="I21" s="2">
+        <v>70.400000000000006</v>
+      </c>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
@@ -1258,7 +1299,9 @@
       <c r="H22" s="2">
         <v>84.1</v>
       </c>
-      <c r="I22" s="2"/>
+      <c r="I22" s="2">
+        <v>84.1</v>
+      </c>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
@@ -1288,7 +1331,9 @@
       <c r="H23" s="2">
         <v>111</v>
       </c>
-      <c r="I23" s="2"/>
+      <c r="I23" s="2">
+        <v>114.2</v>
+      </c>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
@@ -1318,7 +1363,9 @@
       <c r="H24" s="2">
         <v>106.1</v>
       </c>
-      <c r="I24" s="2"/>
+      <c r="I24" s="2">
+        <v>106.1</v>
+      </c>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
@@ -1348,7 +1395,9 @@
       <c r="H25" s="2">
         <v>67.2</v>
       </c>
-      <c r="I25" s="2"/>
+      <c r="I25" s="2">
+        <v>67.8</v>
+      </c>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
@@ -1378,7 +1427,9 @@
       <c r="H26" s="2">
         <v>62.5</v>
       </c>
-      <c r="I26" s="2"/>
+      <c r="I26" s="2">
+        <v>62.3</v>
+      </c>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
@@ -1408,7 +1459,9 @@
       <c r="H27" s="2">
         <v>77.5</v>
       </c>
-      <c r="I27" s="2"/>
+      <c r="I27" s="2">
+        <v>79.7</v>
+      </c>
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
@@ -1436,7 +1489,9 @@
       <c r="H28" s="2">
         <v>74.8</v>
       </c>
-      <c r="I28" s="2"/>
+      <c r="I28" s="2">
+        <v>72.599999999999994</v>
+      </c>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
@@ -1464,7 +1519,9 @@
       <c r="H29" s="2">
         <v>90</v>
       </c>
-      <c r="I29" s="2"/>
+      <c r="I29" s="2">
+        <v>90.1</v>
+      </c>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
@@ -1492,7 +1549,9 @@
       <c r="H30" s="2">
         <v>78</v>
       </c>
-      <c r="I30" s="2"/>
+      <c r="I30" s="2">
+        <v>78</v>
+      </c>
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
@@ -1522,7 +1581,9 @@
       <c r="H31" s="2">
         <v>106.5</v>
       </c>
-      <c r="I31" s="2"/>
+      <c r="I31" s="2">
+        <v>104.8</v>
+      </c>
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
@@ -1552,7 +1613,9 @@
       <c r="H32" s="2">
         <v>74.3</v>
       </c>
-      <c r="I32" s="2"/>
+      <c r="I32" s="2">
+        <v>74.8</v>
+      </c>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
@@ -1582,7 +1645,9 @@
       <c r="H33" s="2">
         <v>88.2</v>
       </c>
-      <c r="I33" s="2"/>
+      <c r="I33" s="2">
+        <v>88.2</v>
+      </c>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
@@ -1612,7 +1677,9 @@
       <c r="H34" s="2">
         <v>71.5</v>
       </c>
-      <c r="I34" s="2"/>
+      <c r="I34" s="2">
+        <v>71.099999999999994</v>
+      </c>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>
@@ -1642,7 +1709,9 @@
       <c r="H35" s="2">
         <v>65.2</v>
       </c>
-      <c r="I35" s="2"/>
+      <c r="I35" s="2">
+        <v>64.099999999999994</v>
+      </c>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
       <c r="L35" s="2"/>
@@ -1672,7 +1741,9 @@
       <c r="H36" s="2">
         <v>73</v>
       </c>
-      <c r="I36" s="2"/>
+      <c r="I36" s="2">
+        <v>73.400000000000006</v>
+      </c>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
@@ -1702,7 +1773,9 @@
       <c r="H37" s="2">
         <v>83.3</v>
       </c>
-      <c r="I37" s="2"/>
+      <c r="I37" s="2">
+        <v>83</v>
+      </c>
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
@@ -1730,7 +1803,9 @@
       <c r="H38" s="3">
         <v>89.4</v>
       </c>
-      <c r="I38" s="3"/>
+      <c r="I38" s="3">
+        <v>89.4</v>
+      </c>
       <c r="J38" s="3"/>
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
@@ -1758,7 +1833,9 @@
       <c r="H39" s="3">
         <v>79.599999999999994</v>
       </c>
-      <c r="I39" s="3"/>
+      <c r="I39" s="3">
+        <v>79.599999999999994</v>
+      </c>
       <c r="J39" s="3"/>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
@@ -1786,7 +1863,9 @@
       <c r="H40" s="3">
         <v>93.6</v>
       </c>
-      <c r="I40" s="3"/>
+      <c r="I40" s="3">
+        <v>93.6</v>
+      </c>
       <c r="J40" s="3"/>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
@@ -1814,7 +1893,9 @@
       <c r="H41" s="3">
         <v>94.8</v>
       </c>
-      <c r="I41" s="3"/>
+      <c r="I41" s="3">
+        <v>94.8</v>
+      </c>
       <c r="J41" s="3"/>
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
@@ -1844,7 +1925,9 @@
       <c r="H42" s="3">
         <v>71.3</v>
       </c>
-      <c r="I42" s="3"/>
+      <c r="I42" s="3">
+        <v>71.2</v>
+      </c>
       <c r="J42" s="3"/>
       <c r="K42" s="3"/>
       <c r="L42" s="3"/>

</xml_diff>

<commit_message>
V5 release: Hall of Fame and Top5 Race
</commit_message>
<xml_diff>
--- a/public/data/BMI ranking raw data.xlsx
+++ b/public/data/BMI ranking raw data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\bmi-ranking-app\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F1035B7-1088-4179-AD91-01392FE42341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BEA574F-C2C8-4EF0-B385-1732628D35FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BD8AD891-FD33-4205-9BBF-5D5C3ED867CE}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="55">
   <si>
     <t>名字</t>
   </si>
@@ -196,9 +196,6 @@
   <si>
     <t>F</t>
     <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>*</t>
   </si>
 </sst>
 </file>
@@ -330,9 +327,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 佈景主題">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 主題">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -370,7 +367,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -476,7 +473,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -618,7 +615,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -728,7 +725,9 @@
       <c r="I3" s="2">
         <v>65.7</v>
       </c>
-      <c r="J3" s="2"/>
+      <c r="J3" s="2">
+        <v>65.900000000000006</v>
+      </c>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
     </row>
@@ -758,7 +757,9 @@
       <c r="I4" s="2">
         <v>68</v>
       </c>
-      <c r="J4" s="2"/>
+      <c r="J4" s="2">
+        <v>67.8</v>
+      </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
@@ -790,7 +791,9 @@
       <c r="I5" s="2">
         <v>73.7</v>
       </c>
-      <c r="J5" s="2"/>
+      <c r="J5" s="2">
+        <v>73.8</v>
+      </c>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
     </row>
@@ -820,7 +823,9 @@
       <c r="I6" s="2">
         <v>78.599999999999994</v>
       </c>
-      <c r="J6" s="2"/>
+      <c r="J6" s="2">
+        <v>78.599999999999994</v>
+      </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
     </row>
@@ -852,7 +857,9 @@
       <c r="I7" s="2">
         <v>67.8</v>
       </c>
-      <c r="J7" s="2"/>
+      <c r="J7" s="2">
+        <v>67.099999999999994</v>
+      </c>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
     </row>
@@ -884,7 +891,9 @@
       <c r="I8" s="2">
         <v>91.7</v>
       </c>
-      <c r="J8" s="2"/>
+      <c r="J8" s="2">
+        <v>91.7</v>
+      </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
     </row>
@@ -916,7 +925,9 @@
       <c r="I9" s="2">
         <v>85.2</v>
       </c>
-      <c r="J9" s="2"/>
+      <c r="J9" s="2">
+        <v>85.2</v>
+      </c>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
     </row>
@@ -946,7 +957,9 @@
       <c r="I10" s="2">
         <v>70.7</v>
       </c>
-      <c r="J10" s="2"/>
+      <c r="J10" s="2">
+        <v>70.7</v>
+      </c>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
     </row>
@@ -976,7 +989,9 @@
       <c r="I11" s="2">
         <v>138</v>
       </c>
-      <c r="J11" s="2"/>
+      <c r="J11" s="2">
+        <v>138</v>
+      </c>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
     </row>
@@ -993,9 +1008,7 @@
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
       <c r="H12" s="2"/>
-      <c r="I12" s="2" t="s">
-        <v>55</v>
-      </c>
+      <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
@@ -1013,9 +1026,7 @@
       <c r="F13" s="6"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
-      <c r="I13" s="2" t="s">
-        <v>55</v>
-      </c>
+      <c r="I13" s="2"/>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
@@ -1048,7 +1059,9 @@
       <c r="I14" s="2">
         <v>82.5</v>
       </c>
-      <c r="J14" s="2"/>
+      <c r="J14" s="2">
+        <v>82.3</v>
+      </c>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
     </row>
@@ -1080,7 +1093,9 @@
       <c r="I15" s="2">
         <v>59.2</v>
       </c>
-      <c r="J15" s="2"/>
+      <c r="J15" s="2">
+        <v>57.1</v>
+      </c>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
     </row>
@@ -1112,7 +1127,9 @@
       <c r="I16" s="2">
         <v>79</v>
       </c>
-      <c r="J16" s="2"/>
+      <c r="J16" s="2">
+        <v>78.3</v>
+      </c>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
     </row>
@@ -1144,7 +1161,9 @@
       <c r="I17" s="2">
         <v>93.9</v>
       </c>
-      <c r="J17" s="2"/>
+      <c r="J17" s="2">
+        <v>93.9</v>
+      </c>
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
     </row>
@@ -1176,7 +1195,9 @@
       <c r="I18" s="2">
         <v>87.9</v>
       </c>
-      <c r="J18" s="2"/>
+      <c r="J18" s="2">
+        <v>88.3</v>
+      </c>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
     </row>
@@ -1208,7 +1229,9 @@
       <c r="I19" s="2">
         <v>87</v>
       </c>
-      <c r="J19" s="2"/>
+      <c r="J19" s="2">
+        <v>87.1</v>
+      </c>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
     </row>
@@ -1240,7 +1263,9 @@
       <c r="I20" s="2">
         <v>84.9</v>
       </c>
-      <c r="J20" s="2"/>
+      <c r="J20" s="2">
+        <v>84.4</v>
+      </c>
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
     </row>
@@ -1270,7 +1295,9 @@
       <c r="I21" s="2">
         <v>70.400000000000006</v>
       </c>
-      <c r="J21" s="2"/>
+      <c r="J21" s="2">
+        <v>70.2</v>
+      </c>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
     </row>
@@ -1302,7 +1329,9 @@
       <c r="I22" s="2">
         <v>84.1</v>
       </c>
-      <c r="J22" s="2"/>
+      <c r="J22" s="2">
+        <v>85.4</v>
+      </c>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
     </row>
@@ -1334,7 +1363,9 @@
       <c r="I23" s="2">
         <v>114.2</v>
       </c>
-      <c r="J23" s="2"/>
+      <c r="J23" s="2">
+        <v>113.9</v>
+      </c>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
     </row>
@@ -1366,7 +1397,9 @@
       <c r="I24" s="2">
         <v>106.1</v>
       </c>
-      <c r="J24" s="2"/>
+      <c r="J24" s="2">
+        <v>106.1</v>
+      </c>
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
     </row>
@@ -1398,7 +1431,9 @@
       <c r="I25" s="2">
         <v>67.8</v>
       </c>
-      <c r="J25" s="2"/>
+      <c r="J25" s="2">
+        <v>68.400000000000006</v>
+      </c>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
     </row>
@@ -1430,7 +1465,9 @@
       <c r="I26" s="2">
         <v>62.3</v>
       </c>
-      <c r="J26" s="2"/>
+      <c r="J26" s="2">
+        <v>62.3</v>
+      </c>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
     </row>
@@ -1462,7 +1499,9 @@
       <c r="I27" s="2">
         <v>79.7</v>
       </c>
-      <c r="J27" s="2"/>
+      <c r="J27" s="2">
+        <v>79.099999999999994</v>
+      </c>
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
     </row>
@@ -1492,7 +1531,9 @@
       <c r="I28" s="2">
         <v>72.599999999999994</v>
       </c>
-      <c r="J28" s="2"/>
+      <c r="J28" s="2">
+        <v>72.599999999999994</v>
+      </c>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
     </row>
@@ -1522,7 +1563,9 @@
       <c r="I29" s="2">
         <v>90.1</v>
       </c>
-      <c r="J29" s="2"/>
+      <c r="J29" s="2">
+        <v>90.1</v>
+      </c>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
     </row>
@@ -1552,7 +1595,9 @@
       <c r="I30" s="2">
         <v>78</v>
       </c>
-      <c r="J30" s="2"/>
+      <c r="J30" s="2">
+        <v>78</v>
+      </c>
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
     </row>
@@ -1584,7 +1629,9 @@
       <c r="I31" s="2">
         <v>104.8</v>
       </c>
-      <c r="J31" s="2"/>
+      <c r="J31" s="2">
+        <v>104.4</v>
+      </c>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
     </row>
@@ -1616,7 +1663,9 @@
       <c r="I32" s="2">
         <v>74.8</v>
       </c>
-      <c r="J32" s="2"/>
+      <c r="J32" s="2">
+        <v>74.3</v>
+      </c>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
     </row>
@@ -1648,7 +1697,9 @@
       <c r="I33" s="2">
         <v>88.2</v>
       </c>
-      <c r="J33" s="2"/>
+      <c r="J33" s="2">
+        <v>88.2</v>
+      </c>
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
     </row>
@@ -1680,7 +1731,9 @@
       <c r="I34" s="2">
         <v>71.099999999999994</v>
       </c>
-      <c r="J34" s="2"/>
+      <c r="J34" s="2">
+        <v>71.099999999999994</v>
+      </c>
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>
     </row>
@@ -1712,7 +1765,9 @@
       <c r="I35" s="2">
         <v>64.099999999999994</v>
       </c>
-      <c r="J35" s="2"/>
+      <c r="J35" s="2">
+        <v>65.599999999999994</v>
+      </c>
       <c r="K35" s="2"/>
       <c r="L35" s="2"/>
     </row>
@@ -1744,7 +1799,9 @@
       <c r="I36" s="2">
         <v>73.400000000000006</v>
       </c>
-      <c r="J36" s="2"/>
+      <c r="J36" s="2">
+        <v>73.3</v>
+      </c>
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
     </row>
@@ -1776,7 +1833,9 @@
       <c r="I37" s="2">
         <v>83</v>
       </c>
-      <c r="J37" s="2"/>
+      <c r="J37" s="2">
+        <v>82.3</v>
+      </c>
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
     </row>
@@ -1806,7 +1865,9 @@
       <c r="I38" s="3">
         <v>89.4</v>
       </c>
-      <c r="J38" s="3"/>
+      <c r="J38" s="3">
+        <v>89.4</v>
+      </c>
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
     </row>
@@ -1836,7 +1897,9 @@
       <c r="I39" s="3">
         <v>79.599999999999994</v>
       </c>
-      <c r="J39" s="3"/>
+      <c r="J39" s="3">
+        <v>79.599999999999994</v>
+      </c>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
     </row>
@@ -1866,7 +1929,9 @@
       <c r="I40" s="3">
         <v>93.6</v>
       </c>
-      <c r="J40" s="3"/>
+      <c r="J40" s="3">
+        <v>93.6</v>
+      </c>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
     </row>
@@ -1896,7 +1961,9 @@
       <c r="I41" s="3">
         <v>94.8</v>
       </c>
-      <c r="J41" s="3"/>
+      <c r="J41" s="3">
+        <v>94.8</v>
+      </c>
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
     </row>
@@ -1928,7 +1995,9 @@
       <c r="I42" s="3">
         <v>71.2</v>
       </c>
-      <c r="J42" s="3"/>
+      <c r="J42" s="3">
+        <v>71.599999999999994</v>
+      </c>
       <c r="K42" s="3"/>
       <c r="L42" s="3"/>
     </row>

</xml_diff>